<commit_message>
Hybrid categorisation with provenance, rule audit, Streamlit demo
- Merchant rules (kubera/rules.py, ~30 unmistakable German merchants)
  decide first; Gemini handles everything else. Every row records who
  decided it in the new "Categorised By" column (rule, own-account rule,
  gemini, or empty = needs review).
- `kubera audit-rules` asks Gemini about every rule-decided text and
  reports the agreement rate, so the rules are measured, not assumed.
- Streamlit demo (demo/app.py): upload a statement or use the synthetic
  sample; shows each booking, its category and the deciding method,
  spending by category and recurring payments. Gemini is capped per upload
  and per day; uploads live in a temp folder and results are never shared
  between visitors.
- Richer synthetic sample (15 bookings, rule and Gemini cases).
- SQL: "Categorised By" column (+ migration). 40 tests incl. the demo.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/barclays_demo.xlsx
+++ b/examples/barclays_demo.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,7 +452,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>-342,17</t>
+          <t>-512,40</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -576,17 +576,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>01.05.2025</t>
+          <t>16.04.2025</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>NETFLIX.COM</t>
+          <t>Fahrradladen Meier Reparatur</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-13,99</t>
+          <t>-64,00</t>
         </is>
       </c>
     </row>
@@ -598,17 +598,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>04.05.2025</t>
+          <t>22.04.2025</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>REWE Markt Erlangen</t>
+          <t>Stadtbibliothek Erlangen Jahresgebuehr</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>-61,05</t>
+          <t>-25,00</t>
         </is>
       </c>
     </row>
@@ -620,17 +620,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>15.05.2025</t>
+          <t>01.05.2025</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Gutschrift Zahlung</t>
+          <t>NETFLIX.COM</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>250,00</t>
+          <t>-13,99</t>
         </is>
       </c>
     </row>
@@ -642,17 +642,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>01.06.2025</t>
+          <t>04.05.2025</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>NETFLIX.COM</t>
+          <t>REWE Markt Erlangen</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>-13,99</t>
+          <t>-61,05</t>
         </is>
       </c>
     </row>
@@ -664,17 +664,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06.06.2025</t>
+          <t>08.05.2025</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Amazon EU</t>
+          <t>Physiotherapie am Markt</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>-89,99</t>
+          <t>-48,00</t>
         </is>
       </c>
     </row>
@@ -686,17 +686,127 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
+          <t>15.05.2025</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Gutschrift Zahlung</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>250,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>R11</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>01.06.2025</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>NETFLIX.COM</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>-13,99</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>R12</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
           <t>06.06.2025</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>Amazon EU</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>-89,99</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>R13</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>06.06.2025</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Amazon EU</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>-89,99</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>R14</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>11.06.2025</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Zahnarztpraxis Dr. Huber</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>-120,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>R15</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>18.06.2025</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Biergarten Entla's Keller</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>-32,80</t>
         </is>
       </c>
     </row>

</xml_diff>